<commit_message>
Features/skilltree - fix (#32)
* 스킬노드 UI에 상태값 반영, 자식 노드 상태값 변경 반영 안 되는 문제 수정

* 스킬 노드 상태 최초 초기화

* 잠금 아이콘 추가

* 스킬트리 테스트용 레벨 게임모드 설정

* 스킬트리 상호 배타 스킬 로직 적용, SkillRow 텍스트 Tid 사용하도록 수정

* 생성 시점 수정 중
</commit_message>
<xml_diff>
--- a/BADesign/Excel/SkillTree.xlsx
+++ b/BADesign/Excel/SkillTree.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -28,16 +28,16 @@
     <t xml:space="preserve">SkillTid</t>
   </si>
   <si>
-    <t xml:space="preserve">SkillName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
+    <t xml:space="preserve">설명</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TextTid</t>
   </si>
   <si>
     <t xml:space="preserve">Prerequisites</t>
   </si>
   <si>
-    <t xml:space="preserve">ExclusiveGroupId</t>
+    <t xml:space="preserve">ExclusiveSkills</t>
   </si>
   <si>
     <t xml:space="preserve">bIsDefaultSkill</t>
@@ -88,16 +88,25 @@
     <t xml:space="preserve">불 속성 강화</t>
   </si>
   <si>
+    <t xml:space="preserve">7,8</t>
+  </si>
+  <si>
     <t xml:space="preserve">/Game/UI/SkillTree/Skill_Icon/Img_fire-enchant-_6_.Img_fire-enchant-_6_</t>
   </si>
   <si>
     <t xml:space="preserve">얼음 속성 강화</t>
   </si>
   <si>
+    <t xml:space="preserve">6,8</t>
+  </si>
+  <si>
     <t xml:space="preserve">/Game/UI/SkillTree/Skill_Icon/Img_ice-enchant-_7_.Img_ice-enchant-_7_</t>
   </si>
   <si>
     <t xml:space="preserve">그냥 강화</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,7</t>
   </si>
   <si>
     <t xml:space="preserve">/Game/UI/SkillTree/Skill_Icon/Img_No-enchant-_8_.Img_No-enchant-_8_</t>
@@ -298,7 +307,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -321,6 +330,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -509,7 +522,9 @@
   <dimension ref="A1:K24"/>
   <sheetFormatPr defaultColWidth="12.67578125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="12.67"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.66"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="12.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.81"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.91"/>
@@ -524,7 +539,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D1" s="2" t="n">
         <v>1</v>
@@ -592,7 +607,9 @@
       <c r="C3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="D3" s="4" t="n">
+        <v>33001</v>
+      </c>
       <c r="E3" s="4"/>
       <c r="F3" s="5"/>
       <c r="G3" s="4" t="n">
@@ -619,7 +636,9 @@
       <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="4" t="n">
+        <v>33002</v>
+      </c>
       <c r="E4" s="4"/>
       <c r="F4" s="5"/>
       <c r="G4" s="4" t="n">
@@ -645,6 +664,9 @@
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="D5" s="1" t="n">
+        <v>33003</v>
+      </c>
       <c r="G5" s="1" t="n">
         <v>1</v>
       </c>
@@ -668,6 +690,9 @@
       <c r="C6" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="D6" s="4" t="n">
+        <v>33004</v>
+      </c>
       <c r="G6" s="1" t="n">
         <v>1</v>
       </c>
@@ -691,6 +716,9 @@
       <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="D7" s="4" t="n">
+        <v>33005</v>
+      </c>
       <c r="G7" s="1" t="n">
         <v>1</v>
       </c>
@@ -714,17 +742,20 @@
       <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="D8" s="1" t="n">
+        <v>33006</v>
+      </c>
       <c r="E8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="1" t="n">
-        <v>18</v>
+      <c r="F8" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J8" s="1" t="n">
         <v>180</v>
@@ -738,19 +769,22 @@
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>33007</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="1" t="n">
-        <v>18</v>
+      <c r="F9" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>300</v>
@@ -764,19 +798,22 @@
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>33008</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="1" t="n">
-        <v>18</v>
+      <c r="F10" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="H10" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>420</v>
@@ -790,7 +827,10 @@
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>33009</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>6</v>
@@ -799,7 +839,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>180</v>
@@ -813,16 +853,19 @@
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>33010</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H12" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J12" s="1" t="n">
         <v>450</v>
@@ -836,7 +879,10 @@
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>33011</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>1</v>
@@ -845,7 +891,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J13" s="1" t="n">
         <v>120</v>
@@ -859,7 +905,10 @@
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>33012</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>11</v>
@@ -868,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J14" s="1" t="n">
         <v>120</v>
@@ -882,7 +931,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>33013</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>3</v>
@@ -891,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="J15" s="1" t="n">
         <v>700</v>
@@ -905,7 +957,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>33014</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>13</v>
@@ -914,7 +969,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="J16" s="1" t="n">
         <v>700</v>
@@ -928,16 +983,19 @@
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>33015</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J17" s="1" t="n">
         <v>1050</v>
@@ -951,7 +1009,10 @@
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>33016</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>15</v>
@@ -960,7 +1021,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="J18" s="1" t="n">
         <v>1050</v>
@@ -974,7 +1035,10 @@
         <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>33017</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>4</v>
@@ -983,7 +1047,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="J19" s="1" t="n">
         <v>1200</v>
@@ -997,7 +1061,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>33018</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>5</v>
@@ -1006,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J20" s="1" t="n">
         <v>1400</v>
@@ -1020,7 +1087,10 @@
         <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>33019</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>5</v>
@@ -1028,8 +1098,8 @@
       <c r="H21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="0" t="s">
-        <v>50</v>
+      <c r="I21" s="6" t="s">
+        <v>53</v>
       </c>
       <c r="J21" s="1" t="n">
         <v>1600</v>
@@ -1043,16 +1113,19 @@
         <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>33020</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="J22" s="1" t="n">
         <v>450</v>
@@ -1066,16 +1139,19 @@
         <v>21</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>33021</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>350</v>

</xml_diff>

<commit_message>
Features/skill apply stat (#85)
* 스탯 변경 스킬 구현

* 가드 시 대미지 감소율 스탯컴포넌트와 연결

* Generate Table
</commit_message>
<xml_diff>
--- a/BADesign/Excel/SkillTree.xlsx
+++ b/BADesign/Excel/SkillTree.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="81">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -221,6 +221,12 @@
     <t xml:space="preserve">Value</t>
   </si>
   <si>
+    <t xml:space="preserve">예상 결과</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reset</t>
+  </si>
+  <si>
     <t xml:space="preserve">Element</t>
   </si>
   <si>
@@ -233,10 +239,28 @@
     <t xml:space="preserve">AttackSpeed</t>
   </si>
   <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
     <t xml:space="preserve">MovesetKey</t>
   </si>
   <si>
     <t xml:space="preserve">Dash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxStamina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StaminaRecovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가드 시 피해 감소율 증가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본값 0.5 * 1.5 = 0.75</t>
   </si>
   <si>
     <t xml:space="preserve">Etc</t>
@@ -391,7 +415,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -421,7 +445,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -430,10 +454,6 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -457,7 +477,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1447,19 +1467,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultColWidth="12.67578125" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K18"/>
+  <sheetFormatPr defaultColWidth="12.67578125" defaultRowHeight="16.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="7.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="8.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="22.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="26.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="11.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="17.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="18.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="7.12"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="7" width="12.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="23.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="6.94"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="7" width="12.67"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1478,8 +1500,14 @@
       <c r="F1" s="8" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G1" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9"/>
       <c r="B2" s="9" t="s">
         <v>1</v>
@@ -1496,240 +1524,238 @@
       <c r="F2" s="9" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11" t="n">
+      <c r="G2" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11" t="n">
+      <c r="D3" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11" t="n">
+      <c r="D4" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11" t="n">
+      <c r="D5" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11" t="n">
+      <c r="D6" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11" t="n">
+      <c r="D7" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="D8" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11" t="n">
+    </row>
+    <row r="10" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" s="10" t="s">
+      <c r="D10" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11" t="n">
-        <v>14</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11" t="n">
+      <c r="E12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11" t="n">
+      <c r="D13" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11" t="n">
+      <c r="C14" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11" t="n">
+      <c r="D15" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11" t="n">
+      <c r="D16" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11" t="n">
+      <c r="D17" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
+      <c r="D18" s="13" t="s">
+        <v>69</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Features/skill apply element (#103)
* 스킬트리 엑셀

* 무기애셋 Pivot 변경버전

* 무기 효과를 위한 나이아가라 컴포넌트 추가

* 컴포넌트로 분리, 리셋 함수 추가

* 무기 효과, 트레일 효과 분리 가능하도록 설정

* 무기 vfx 적용

* ANS_Collision에서 트레일 켜고 꺼지도록 수정

* CDO 오류 수정

* 이름 및 설명 수정

* 무기 vfx 애셋 추가

* 트레일 VFX 애셋

* 애셋 파라미터 및 엑셀 수정
</commit_message>
<xml_diff>
--- a/BADesign/Excel/SkillTree.xlsx
+++ b/BADesign/Excel/SkillTree.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="7"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="91">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -212,24 +212,57 @@
     <t xml:space="preserve">/Game/UI/SkillTree/Skill_Icon/Img_Charged-Attack.Img_Charged-Attack</t>
   </si>
   <si>
+    <t xml:space="preserve">스킬 설명설명</t>
+  </si>
+  <si>
     <t xml:space="preserve">ApplyType</t>
   </si>
   <si>
     <t xml:space="preserve">Target</t>
   </si>
   <si>
+    <t xml:space="preserve">값 설명</t>
+  </si>
+  <si>
     <t xml:space="preserve">Value</t>
   </si>
   <si>
-    <t xml:space="preserve">예상 결과</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reset</t>
+    <t xml:space="preserve">Value2</t>
   </si>
   <si>
     <t xml:space="preserve">Element</t>
   </si>
   <si>
+    <t xml:space="preserve">WeaponVFX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value: 무기 VFX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Weapon/MeleeWeaponAura_VFX/VFX/V4/NS_StylizedWeapon_V4_05.NS_StylizedWeapon_V4_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Trail/SwordTrailVFX/VFX/NS_Trail_03.NS_Trail_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value2: 트레일 VFX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Trail/SlashTrailElemental/Niagara/Sword/NS_Sword_Ice.NS_Sword_Ice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Trail/SlashTrailElemental/Niagara/SlashTrail/NS_SlashTrail_Ice.NS_SlashTrail_Ice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Weapon/MeleeWeaponAura_VFX/VFX/V3/NS_StylizedWeapon_V3_09.NS_StylizedWeapon_V3_09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Game/Assets/WeaponVFX/Trail/SwordTrailVFX/VFX/NS_Trail_12.NS_Trail_12</t>
+  </si>
+  <si>
     <t xml:space="preserve">Action</t>
   </si>
   <si>
@@ -239,12 +272,12 @@
     <t xml:space="preserve">AttackSpeed</t>
   </si>
   <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
     <t xml:space="preserve">MovesetKey</t>
   </si>
   <si>
+    <t xml:space="preserve">Moveset 키 추가</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dash</t>
   </si>
   <si>
@@ -258,9 +291,6 @@
   </si>
   <si>
     <t xml:space="preserve">Guard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기본값 0.5 * 1.5 = 0.75</t>
   </si>
   <si>
     <t xml:space="preserve">Etc</t>
@@ -284,16 +314,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="9"/>
@@ -330,7 +363,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -346,6 +379,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCCCCCC"/>
+        <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE8CB"/>
         <bgColor rgb="FFDDDDDD"/>
       </patternFill>
     </fill>
@@ -415,7 +454,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -448,39 +487,59 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -529,7 +588,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFDDE8CB"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -564,37 +623,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1467,294 +1526,323 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="12.67578125" defaultRowHeight="16.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="7.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="8.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="26.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="11.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="18.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="7.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="23.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="6.94"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="7" width="12.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="6.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="8.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="25.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="11.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="17.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="22.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="7" width="28.07"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="9" style="7" width="12.67"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="19" style="7" width="12.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="n">
+      <c r="B1" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E1" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F1" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G1" s="7" t="n">
+      <c r="D1" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H1" s="7" t="n">
-        <v>0</v>
+      <c r="G1" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="D2" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="E2" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="F2" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="G2" s="11" t="s">
         <v>67</v>
       </c>
+      <c r="H2" s="11" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="12" t="s">
-        <v>68</v>
+      <c r="D3" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="12" t="s">
-        <v>68</v>
+      <c r="D4" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>68</v>
+      <c r="D5" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>69</v>
+      <c r="D6" s="18" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>69</v>
+      <c r="D7" s="18" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>70</v>
+      <c r="D8" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <v>1.2</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="13" t="s">
-        <v>69</v>
+      <c r="D9" s="18" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>69</v>
+      <c r="D10" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>72</v>
+        <v>83</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>69</v>
+      <c r="D11" s="18" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="C12" s="11" t="s">
+      <c r="B12" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="14" t="s">
-        <v>70</v>
+      <c r="D12" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F12" s="7" t="n">
+        <v>86</v>
+      </c>
+      <c r="G12" s="7" t="n">
         <v>1.2</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>70</v>
+      <c r="D13" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F13" s="7" t="n">
+        <v>87</v>
+      </c>
+      <c r="G13" s="7" t="n">
         <v>1.2</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="19.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>70</v>
+      <c r="C14" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="7" t="n">
+        <v>89</v>
+      </c>
+      <c r="G14" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="18" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16" s="16" t="s">
+    <row r="18" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="16.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>